<commit_message>
The SoIB mapping file, main file with and without the categories and summary file have been updated to reflect changes in the taxonomy of 3 species (Demoiselle crane, White tern and Striated heron) and to remove a duplicate entry of the Eastern red-rumped swallow. Some scripts to compare trend outputs and priorities
</commit_message>
<xml_diff>
--- a/01_analyses_full/results/SoIB_summaries.xlsx
+++ b/01_analyses_full/results/SoIB_summaries.xlsx
@@ -407,16 +407,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C2">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D2">
-        <v>16.7</v>
+        <v>15.6</v>
       </c>
       <c r="E2">
-        <v>11.8</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="3">
@@ -426,16 +426,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C3">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D3">
-        <v>25.9</v>
+        <v>24.5</v>
       </c>
       <c r="E3">
-        <v>26</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="4">
@@ -445,16 +445,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C4">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D4">
-        <v>32.5</v>
+        <v>34</v>
       </c>
       <c r="E4">
-        <v>48.3</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="5">
@@ -464,16 +464,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C5">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="E5">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="6">
@@ -483,16 +483,16 @@
         </is>
       </c>
       <c r="B6">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6">
-        <v>13.6</v>
+        <v>15.1</v>
       </c>
       <c r="E6">
-        <v>8.300000000000001</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="7">
@@ -502,10 +502,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>298</v>
+        <v>318</v>
       </c>
       <c r="C7">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="8">
@@ -515,10 +515,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="C8">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -834,10 +834,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3">
-        <v>17.5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -886,10 +886,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C7">
-        <v>22.5</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="8">
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>23.8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -1158,7 +1158,7 @@
         <v>32</v>
       </c>
       <c r="D6">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="7">
@@ -1173,10 +1173,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D7">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="8">
@@ -1406,10 +1406,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D7">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="8">
@@ -1427,7 +1427,7 @@
         <v>81</v>
       </c>
       <c r="D8">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="9">
@@ -1636,10 +1636,10 @@
         <v>273</v>
       </c>
       <c r="D6">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E6">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="7">
@@ -1674,10 +1674,10 @@
         <v>323</v>
       </c>
       <c r="D8">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E8">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
   </sheetData>
@@ -1786,10 +1786,10 @@
         <v>11.1</v>
       </c>
       <c r="C6">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="D6">
-        <v>54.2</v>
+        <v>54.1</v>
       </c>
     </row>
     <row r="7">
@@ -2173,10 +2173,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C7">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
     </row>
   </sheetData>
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
   </sheetData>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="3">
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="C3">
-        <v>228</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4">
@@ -2435,7 +2435,7 @@
         <v>651</v>
       </c>
       <c r="C4">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
   </sheetData>
@@ -2455,7 +2455,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2488,51 +2488,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Trend Different</t>
+          <t>Trend New</t>
         </is>
       </c>
       <c r="B2">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>24.3</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Trend Different</t>
         </is>
       </c>
       <c r="B3">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C3">
-        <v>36.9</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>40</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>38</v>
+      </c>
+      <c r="C4">
+        <v>36.9</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>IUCN</t>
         </is>
       </c>
-      <c r="B4">
-        <v>40</v>
-      </c>
-      <c r="C4">
-        <v>38.8</v>
-      </c>
-      <c r="D4">
+      <c r="B5">
+        <v>38</v>
+      </c>
+      <c r="C5">
+        <v>36.9</v>
+      </c>
+      <c r="D5">
         <v>3</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>60</v>
       </c>
     </row>
@@ -2652,10 +2665,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D6">
-        <v>96.2</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -2846,7 +2859,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D6">
         <v>76.7</v>
@@ -3050,10 +3063,10 @@
         <v>215</v>
       </c>
       <c r="D6">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E6">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="7">
@@ -3088,10 +3101,10 @@
         <v>286</v>
       </c>
       <c r="D8">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="E8">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
   </sheetData>
@@ -3203,7 +3216,7 @@
         <v>27.4</v>
       </c>
       <c r="D6">
-        <v>69</v>
+        <v>68.90000000000001</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
After all the final runs for 2026
</commit_message>
<xml_diff>
--- a/01_analyses_full/results/SoIB_summaries.xlsx
+++ b/01_analyses_full/results/SoIB_summaries.xlsx
@@ -407,16 +407,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>33</v>
+        <v>118</v>
       </c>
       <c r="C2">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="D2">
-        <v>15.6</v>
+        <v>34.5</v>
       </c>
       <c r="E2">
-        <v>12.9</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3">
@@ -426,16 +426,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="C3">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="D3">
-        <v>24.5</v>
+        <v>31.9</v>
       </c>
       <c r="E3">
-        <v>25.7</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="4">
@@ -445,16 +445,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="C4">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D4">
-        <v>34</v>
+        <v>17.8</v>
       </c>
       <c r="E4">
-        <v>49.3</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="5">
@@ -464,16 +464,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D5">
-        <v>10.8</v>
+        <v>7.6</v>
       </c>
       <c r="E5">
-        <v>4.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="6">
@@ -483,16 +483,16 @@
         </is>
       </c>
       <c r="B6">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C6">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>15.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E6">
-        <v>7.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -502,10 +502,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>318</v>
+        <v>183</v>
       </c>
       <c r="C7">
-        <v>371</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8">
@@ -515,10 +515,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="C8">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -575,19 +575,19 @@
         </is>
       </c>
       <c r="B2">
+        <v>12.6</v>
+      </c>
+      <c r="C2">
+        <v>10.7</v>
+      </c>
+      <c r="D2">
+        <v>29.1</v>
+      </c>
+      <c r="E2">
         <v>14.6</v>
       </c>
-      <c r="C2">
-        <v>12.6</v>
-      </c>
-      <c r="D2">
-        <v>31.1</v>
-      </c>
-      <c r="E2">
-        <v>13.6</v>
-      </c>
       <c r="F2">
-        <v>28.2</v>
+        <v>33</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B3">
+        <v>0.8</v>
+      </c>
+      <c r="C3">
         <v>0.3</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
       <c r="D3">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
       <c r="E3">
-        <v>18.9</v>
+        <v>12.4</v>
       </c>
       <c r="F3">
-        <v>75.2</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G3">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="4">
@@ -628,19 +628,19 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D4">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="E4">
-        <v>0.5</v>
+        <v>1.8</v>
       </c>
       <c r="F4">
-        <v>97.8</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G4">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -677,10 +677,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="3">
@@ -690,10 +690,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="4">
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="5">
@@ -716,10 +716,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="6">
@@ -729,10 +729,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="7">
@@ -755,10 +755,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -771,7 +771,7 @@
         <v>2</v>
       </c>
       <c r="C9">
-        <v>40</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="10">
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10">
-        <v>40</v>
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>
@@ -821,10 +821,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C2">
-        <v>16.2</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -834,10 +834,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="4">
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="7">
@@ -886,10 +886,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C7">
-        <v>18.8</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="8">
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="C8">
-        <v>30</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="9">
@@ -912,10 +912,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C9">
-        <v>12.5</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="10">
@@ -928,7 +928,7 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
     </row>
   </sheetData>
@@ -1176,7 +1176,7 @@
         <v>333</v>
       </c>
       <c r="D7">
-        <v>75.5</v>
+        <v>75.7</v>
       </c>
     </row>
     <row r="8">
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="C8">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D8">
-        <v>16.3</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="9">
@@ -1473,10 +1473,10 @@
         </is>
       </c>
       <c r="C11">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D11">
-        <v>22.3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
@@ -1504,10 +1504,10 @@
         </is>
       </c>
       <c r="C13">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13">
-        <v>19.5</v>
+        <v>19.8</v>
       </c>
     </row>
   </sheetData>
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -1601,7 +1601,7 @@
         <v>2</v>
       </c>
       <c r="E4">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -1633,13 +1633,13 @@
         <v>87</v>
       </c>
       <c r="C6">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D6">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="E6">
-        <v>785</v>
+        <v>777</v>
       </c>
     </row>
     <row r="7">
@@ -1655,10 +1655,10 @@
         <v>8</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E7">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1668,16 +1668,16 @@
         </is>
       </c>
       <c r="B8">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C8">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D8">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="E8">
-        <v>942</v>
+        <v>931</v>
       </c>
     </row>
   </sheetData>
@@ -1751,13 +1751,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>85.7</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="C4">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D4">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="5">
@@ -1783,13 +1783,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C6">
-        <v>34.8</v>
+        <v>34.6</v>
       </c>
       <c r="D6">
-        <v>54.1</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="7">
@@ -1802,10 +1802,10 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>53.3</v>
+        <v>61.5</v>
       </c>
       <c r="D7">
-        <v>46.7</v>
+        <v>38.5</v>
       </c>
     </row>
   </sheetData>
@@ -1868,13 +1868,13 @@
         <v>6.2</v>
       </c>
       <c r="D2">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="E2">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="F2">
-        <v>48.9</v>
+        <v>49.2</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1893,13 +1893,13 @@
         <v>0.3</v>
       </c>
       <c r="D3">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E3">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="F3">
-        <v>84.5</v>
+        <v>84.3</v>
       </c>
       <c r="G3">
         <v>2.5</v>
@@ -1924,10 +1924,10 @@
         <v>1.4</v>
       </c>
       <c r="F4">
-        <v>96.40000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="G4">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -2108,10 +2108,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
@@ -2121,10 +2121,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="4">
@@ -2134,10 +2134,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C4">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="5">
@@ -2147,10 +2147,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C5">
-        <v>38.5</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="6">
@@ -2160,10 +2160,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C6">
-        <v>18.7</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="7">
@@ -2173,10 +2173,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C7">
-        <v>16.8</v>
+        <v>15.9</v>
       </c>
     </row>
   </sheetData>
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>286</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>553</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>942</v>
+        <v>931</v>
       </c>
     </row>
     <row r="3">
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="C3">
-        <v>212</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4">
@@ -2432,10 +2432,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>651</v>
+        <v>644</v>
       </c>
       <c r="C4">
-        <v>280</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5">
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>942</v>
+        <v>931</v>
       </c>
     </row>
   </sheetData>
@@ -2492,10 +2492,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C2">
-        <v>1.9</v>
+        <v>12.6</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>58.8</v>
       </c>
     </row>
     <row r="3">
@@ -2505,10 +2511,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C3">
-        <v>24.3</v>
+        <v>18.4</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>11.8</v>
       </c>
     </row>
     <row r="4">
@@ -2518,16 +2530,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C4">
-        <v>36.9</v>
+        <v>34</v>
       </c>
       <c r="D4">
         <v>2</v>
       </c>
       <c r="E4">
-        <v>40</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="5">
@@ -2537,16 +2549,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C5">
-        <v>36.9</v>
+        <v>35</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5">
-        <v>60</v>
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>
@@ -2556,7 +2568,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2593,10 +2605,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D2">
-        <v>55.1</v>
+        <v>48.3</v>
       </c>
     </row>
     <row r="3">
@@ -2611,10 +2623,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>12.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="4">
@@ -2629,20 +2641,15 @@
         </is>
       </c>
       <c r="C4">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="D4">
-        <v>32.6</v>
+        <v>47.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
           <t>High</t>
         </is>
       </c>
@@ -2650,7 +2657,7 @@
         <v>1</v>
       </c>
       <c r="D5">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -2661,14 +2668,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C6">
-        <v>424</v>
+        <v>3</v>
       </c>
       <c r="D6">
-        <v>96.09999999999999</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
@@ -2679,50 +2686,45 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C7">
-        <v>16</v>
+        <v>369</v>
       </c>
       <c r="D7">
-        <v>3.6</v>
+        <v>83.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="D8">
-        <v>1.2</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
           <t>Low</t>
         </is>
       </c>
       <c r="C9">
-        <v>107</v>
+        <v>6</v>
       </c>
       <c r="D9">
-        <v>33.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="10">
@@ -2733,14 +2735,63 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10">
-        <v>212</v>
+        <v>14</v>
       </c>
       <c r="D10">
-        <v>65.59999999999999</v>
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>66</v>
+      </c>
+      <c r="D11">
+        <v>20.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>239</v>
+      </c>
+      <c r="D12">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -2787,10 +2838,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D2">
-        <v>95.09999999999999</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="3">
@@ -2805,10 +2856,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="4">
@@ -2823,10 +2874,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D4">
-        <v>3.9</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="5">
@@ -2841,10 +2892,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6">
@@ -2859,10 +2910,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>424</v>
+        <v>369</v>
       </c>
       <c r="D6">
-        <v>76.7</v>
+        <v>83.7</v>
       </c>
     </row>
     <row r="7">
@@ -2877,10 +2928,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>107</v>
+        <v>66</v>
       </c>
       <c r="D7">
-        <v>19.3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -2895,10 +2946,10 @@
         </is>
       </c>
       <c r="C8">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="D8">
-        <v>20.3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -2913,10 +2964,10 @@
         </is>
       </c>
       <c r="C9">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="D9">
-        <v>5.6</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="10">
@@ -2931,10 +2982,10 @@
         </is>
       </c>
       <c r="C10">
-        <v>212</v>
+        <v>239</v>
       </c>
       <c r="D10">
-        <v>74.09999999999999</v>
+        <v>61.8</v>
       </c>
     </row>
   </sheetData>
@@ -2981,10 +3032,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -3000,13 +3051,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>13</v>
@@ -3019,16 +3070,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>8</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -3038,13 +3089,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E5">
         <v>71</v>
@@ -3057,16 +3108,16 @@
         </is>
       </c>
       <c r="B6">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>215</v>
+        <v>319</v>
       </c>
       <c r="D6">
-        <v>541</v>
+        <v>424</v>
       </c>
       <c r="E6">
-        <v>785</v>
+        <v>777</v>
       </c>
     </row>
     <row r="7">
@@ -3082,10 +3133,10 @@
         <v>8</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E7">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -3098,13 +3149,13 @@
         <v>103</v>
       </c>
       <c r="C8">
-        <v>286</v>
+        <v>387</v>
       </c>
       <c r="D8">
-        <v>553</v>
+        <v>441</v>
       </c>
       <c r="E8">
-        <v>942</v>
+        <v>931</v>
       </c>
     </row>
   </sheetData>
@@ -3146,10 +3197,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>93.8</v>
+        <v>81.2</v>
       </c>
       <c r="C2">
-        <v>6.2</v>
+        <v>18.8</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -3162,13 +3213,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>100</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="4">
@@ -3178,13 +3229,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>76.2</v>
+        <v>73.2</v>
       </c>
       <c r="C4">
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="D4">
-        <v>4.8</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="5">
@@ -3194,13 +3245,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>19.7</v>
+        <v>21.1</v>
       </c>
       <c r="C5">
-        <v>76.09999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="D5">
-        <v>4.2</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="6">
@@ -3210,13 +3261,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="C6">
-        <v>27.4</v>
+        <v>41.1</v>
       </c>
       <c r="D6">
-        <v>68.90000000000001</v>
+        <v>54.6</v>
       </c>
     </row>
     <row r="7">
@@ -3229,10 +3280,10 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>53.3</v>
+        <v>61.5</v>
       </c>
       <c r="D7">
-        <v>46.7</v>
+        <v>38.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>